<commit_message>
update to newest IG
</commit_message>
<xml_diff>
--- a/site/StructureDefinition-KBV-EX-WEST-Patient-Postleitzahl-und-Ort.xlsx
+++ b/site/StructureDefinition-KBV-EX-WEST-Patient-Postleitzahl-und-Ort.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="113">
   <si>
     <t>Property</t>
   </si>
@@ -54,7 +54,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-03-11T11:00:33+01:00</t>
+    <t>2026-03-18T11:15:18+01:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -337,18 +337,30 @@
     <t>Extension.value[x]</t>
   </si>
   <si>
+    <t>Value of extension</t>
+  </si>
+  <si>
     <t>Value of extension - must be one of a constrained set of the data types (see [Extensibility](http://hl7.org/fhir/R4/extensibility.html) for a list).</t>
-  </si>
-  <si>
-    <t>Postleitzahl und Ort in gemeinsamer Angabe</t>
   </si>
   <si>
     <t xml:space="preserve">type:$this}
 </t>
   </si>
   <si>
+    <t>closed</t>
+  </si>
+  <si>
     <t xml:space="preserve">ele-1:All FHIR elements must have a @value or children {hasValue() or (children().count() &gt; id.count())}
 </t>
+  </si>
+  <si>
+    <t>Extension.value[x]:valueString</t>
+  </si>
+  <si>
+    <t>valueString</t>
+  </si>
+  <si>
+    <t>Postleitzahl und Ort in gemeinsamer Angabe</t>
   </si>
 </sst>
 </file>
@@ -660,10 +672,10 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:AK6"/>
+  <dimension ref="A1:AK7"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="16.80078125" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="25.07421875" customWidth="true" bestFit="true"/>
     <col min="2" max="2" width="16.80078125" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="10.8515625" customWidth="true" bestFit="true" hidden="true"/>
     <col min="4" max="4" width="7.6796875" customWidth="true" bestFit="true" hidden="true"/>
@@ -1259,14 +1271,12 @@
         <v>86</v>
       </c>
       <c r="L6" t="s" s="2">
-        <v>80</v>
+        <v>105</v>
       </c>
       <c r="M6" t="s" s="2">
-        <v>105</v>
-      </c>
-      <c r="N6" t="s" s="2">
         <v>106</v>
       </c>
+      <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" t="s" s="2">
         <v>76</v>
@@ -1310,7 +1320,7 @@
         <v>76</v>
       </c>
       <c r="AE6" t="s" s="2">
-        <v>96</v>
+        <v>108</v>
       </c>
       <c r="AF6" t="s" s="2">
         <v>104</v>
@@ -1325,9 +1335,116 @@
         <v>76</v>
       </c>
       <c r="AJ6" t="s" s="2">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="AK6" t="s" s="2">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="2">
+        <v>110</v>
+      </c>
+      <c r="B7" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="C7" t="s" s="2">
+        <v>111</v>
+      </c>
+      <c r="D7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="E7" s="2"/>
+      <c r="F7" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="G7" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="H7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="I7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="J7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="K7" t="s" s="2">
+        <v>86</v>
+      </c>
+      <c r="L7" t="s" s="2">
+        <v>80</v>
+      </c>
+      <c r="M7" t="s" s="2">
+        <v>106</v>
+      </c>
+      <c r="N7" t="s" s="2">
+        <v>112</v>
+      </c>
+      <c r="O7" s="2"/>
+      <c r="P7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Q7" s="2"/>
+      <c r="R7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="S7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="T7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="U7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="V7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="W7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="X7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Y7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="Z7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AA7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AB7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AC7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AD7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AE7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AF7" t="s" s="2">
+        <v>104</v>
+      </c>
+      <c r="AG7" t="s" s="2">
+        <v>77</v>
+      </c>
+      <c r="AH7" t="s" s="2">
+        <v>85</v>
+      </c>
+      <c r="AI7" t="s" s="2">
+        <v>76</v>
+      </c>
+      <c r="AJ7" t="s" s="2">
+        <v>109</v>
+      </c>
+      <c r="AK7" t="s" s="2">
         <v>103</v>
       </c>
     </row>

</xml_diff>